<commit_message>
Rebuild the client pack around the 44 parked services
The pack previously asked the client to confirm 56 drafted services. Their
business profile has since answered most of that, so it now asks only what
is genuinely open.

- "Services to verify" — the 44 parked services, each with what would have
  to be true to advertise it and which group it falls into: a significant
  capability absent from their profile, one needing a named qualified
  person, a plausible extension, or superseded.
- "Services now live" — the 30 published lines, straight from the profile,
  for a quick correctness check rather than a decision.
- The PDF mirrors both, with 44 radio groups and 44 note fields.

Both files carry the corrected short domain.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S17Tp8qvoSXk69wgS8r39a
</commit_message>
<xml_diff>
--- a/handover/INTEGRI-Information-Request.xlsx
+++ b/handover/INTEGRI-Information-Request.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Start here" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Services" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Company details" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="People" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Documents" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Services to verify" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Services now live" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Company details" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="People" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Documents" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -145,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -186,6 +187,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -193,8 +197,8 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -762,28 +766,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The 56 services on your website</t>
+          <t>44 services we have taken OFF your website</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mark each TRUE or FALSE. Anything FALSE comes off the site. Use the note column to reword.</t>
+          <t>These are not in your business profile, so we parked them. Mark each one TRUE if INTEGRI does it, and we will put it back.</t>
         </is>
       </c>
     </row>
@@ -810,12 +815,17 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
+          <t>Why we parked it</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
           <t>TRUE / FALSE</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Your note or rewording</t>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Your note</t>
         </is>
       </c>
     </row>
@@ -832,12 +842,13 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>8 services</t>
+          <t>7 parked</t>
         </is>
       </c>
       <c r="D5" s="13" t="n"/>
       <c r="E5" s="13" t="n"/>
       <c r="F5" s="13" t="n"/>
+      <c r="G5" s="13" t="n"/>
     </row>
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
@@ -856,8 +867,13 @@
           <t>We can investigate internal misconduct, theft or policy breaches inside a client's business and deliver a written report.</t>
         </is>
       </c>
-      <c r="E6" s="18" t="n"/>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>A — Significant capability absent from your profile</t>
+        </is>
+      </c>
       <c r="F6" s="19" t="n"/>
+      <c r="G6" s="20" t="n"/>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
@@ -876,8 +892,13 @@
           <t>We have someone able to investigate fraud, establish how money moved, and document it to an evidentiary standard.</t>
         </is>
       </c>
-      <c r="E7" s="18" t="n"/>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>B — Needs a named, qualified person</t>
+        </is>
+      </c>
       <c r="F7" s="19" t="n"/>
+      <c r="G7" s="20" t="n"/>
     </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
@@ -896,8 +917,13 @@
           <t>We have trained operatives and equipment to run lawful physical surveillance, and to detect surveillance run against a client.</t>
         </is>
       </c>
-      <c r="E8" s="18" t="n"/>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>B — Needs a named, qualified person</t>
+        </is>
+      </c>
       <c r="F8" s="19" t="n"/>
+      <c r="G8" s="20" t="n"/>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
@@ -908,16 +934,21 @@
       <c r="B9" s="15" t="n"/>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Background screening &amp; vetting</t>
+          <t>Insurance claim investigation</t>
         </is>
       </c>
       <c r="D9" s="17" t="inlineStr">
         <is>
-          <t>We can run pre-employment and due-diligence background checks, with the subject's consent where the law requires it.</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="n"/>
+          <t>We take instructions from insurers or brokers to investigate suspect claims and report findings.</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>C — Plausible extension of confirmed work</t>
+        </is>
+      </c>
       <c r="F9" s="19" t="n"/>
+      <c r="G9" s="20" t="n"/>
     </row>
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
@@ -928,16 +959,21 @@
       <c r="B10" s="15" t="n"/>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>Insurance claim investigation</t>
+          <t>Asset tracing &amp; due diligence</t>
         </is>
       </c>
       <c r="D10" s="17" t="inlineStr">
         <is>
-          <t>We take instructions from insurers or brokers to investigate suspect claims and report findings.</t>
-        </is>
-      </c>
-      <c r="E10" s="18" t="n"/>
+          <t>We can trace assets, company interests and directorships, and compile a due-diligence report.</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>C — Plausible extension of confirmed work</t>
+        </is>
+      </c>
       <c r="F10" s="19" t="n"/>
+      <c r="G10" s="20" t="n"/>
     </row>
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
@@ -948,16 +984,21 @@
       <c r="B11" s="15" t="n"/>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>Asset tracing &amp; due diligence</t>
+          <t>Missing persons tracing</t>
         </is>
       </c>
       <c r="D11" s="17" t="inlineStr">
         <is>
-          <t>We can trace assets, company interests and directorships, and compile a due-diligence report.</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="n"/>
+          <t>We take on missing-person and skip-tracing work.</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>D — Superseded or narrow</t>
+        </is>
+      </c>
       <c r="F11" s="19" t="n"/>
+      <c r="G11" s="20" t="n"/>
     </row>
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
@@ -968,1178 +1009,1123 @@
       <c r="B12" s="15" t="n"/>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>Missing persons tracing</t>
+          <t>Matrimonial &amp; domestic enquiry</t>
         </is>
       </c>
       <c r="D12" s="17" t="inlineStr">
         <is>
-          <t>We take on missing-person and skip-tracing work.</t>
-        </is>
-      </c>
-      <c r="E12" s="18" t="n"/>
+          <t>We take on private matrimonial and domestic investigations for individual clients.</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>C — Plausible extension of confirmed work</t>
+        </is>
+      </c>
       <c r="F12" s="19" t="n"/>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>01.8</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="n"/>
-      <c r="C13" s="16" t="inlineStr">
-        <is>
-          <t>Matrimonial &amp; domestic enquiry</t>
-        </is>
-      </c>
-      <c r="D13" s="17" t="inlineStr">
-        <is>
-          <t>We take on private matrimonial and domestic investigations for individual clients.</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="n"/>
-      <c r="F13" s="19" t="n"/>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="G12" s="20" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Forensic Services</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>8 services</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="n"/>
-      <c r="E14" s="13" t="n"/>
-      <c r="F14" s="13" t="n"/>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>8 parked</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="13" t="n"/>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="13" t="n"/>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>02.1</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="n"/>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Crime scene processing &amp; documentation</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>We attend scenes and photograph, document, and recover physical evidence using proper method.</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>B — Needs a named, qualified person</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="20" t="n"/>
     </row>
     <row r="15" ht="34" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>02.1</t>
+          <t>02.2</t>
         </is>
       </c>
       <c r="B15" s="15" t="n"/>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>Crime scene processing &amp; documentation</t>
+          <t>Fingerprint collection &amp; comparison</t>
         </is>
       </c>
       <c r="D15" s="17" t="inlineStr">
         <is>
-          <t>We attend scenes and photograph, document, and recover physical evidence using proper method.</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="n"/>
+          <t>We can BOTH lift latent prints AND have someone competent to compare and identify them. Lifting alone is not enough for this line.</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>B — Needs a named, qualified person</t>
+        </is>
+      </c>
       <c r="F15" s="19" t="n"/>
+      <c r="G15" s="20" t="n"/>
     </row>
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>02.2</t>
+          <t>02.3</t>
         </is>
       </c>
       <c r="B16" s="15" t="n"/>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>Fingerprint collection &amp; comparison</t>
+          <t>Questioned document examination</t>
         </is>
       </c>
       <c r="D16" s="17" t="inlineStr">
         <is>
-          <t>We can BOTH lift latent prints AND have someone competent to compare and identify them. Lifting alone is not enough for this line.</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="n"/>
+          <t>We have a trained document examiner who can examine signatures, handwriting and alterations.</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>B — Needs a named, qualified person</t>
+        </is>
+      </c>
       <c r="F16" s="19" t="n"/>
+      <c r="G16" s="20" t="n"/>
     </row>
     <row r="17" ht="34" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>02.3</t>
+          <t>02.4</t>
         </is>
       </c>
       <c r="B17" s="15" t="n"/>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>Questioned document examination</t>
+          <t>Digital &amp; mobile device forensics</t>
         </is>
       </c>
       <c r="D17" s="17" t="inlineStr">
         <is>
-          <t>We have a trained document examiner who can examine signatures, handwriting and alterations.</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="n"/>
+          <t>We have forensic acquisition tools and a competent examiner who can image and analyse devices defensibly.</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>B — Needs a named, qualified person</t>
+        </is>
+      </c>
       <c r="F17" s="19" t="n"/>
+      <c r="G17" s="20" t="n"/>
     </row>
     <row r="18" ht="34" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>02.4</t>
+          <t>02.5</t>
         </is>
       </c>
       <c r="B18" s="15" t="n"/>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>Digital &amp; mobile device forensics</t>
+          <t>Forensic auditing</t>
         </is>
       </c>
       <c r="D18" s="17" t="inlineStr">
         <is>
-          <t>We have forensic acquisition tools and a competent examiner who can image and analyse devices defensibly.</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="n"/>
+          <t>We have someone with an accounting or audit qualification able to conduct a forensic audit.</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>B — Needs a named, qualified person</t>
+        </is>
+      </c>
       <c r="F18" s="19" t="n"/>
+      <c r="G18" s="20" t="n"/>
     </row>
     <row r="19" ht="34" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>02.5</t>
+          <t>02.6</t>
         </is>
       </c>
       <c r="B19" s="15" t="n"/>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>Forensic auditing</t>
+          <t>Evidence handling &amp; chain of custody</t>
         </is>
       </c>
       <c r="D19" s="17" t="inlineStr">
         <is>
-          <t>We have someone with an accounting or audit qualification able to conduct a forensic audit.</t>
-        </is>
-      </c>
-      <c r="E19" s="18" t="n"/>
+          <t>We operate a documented chain-of-custody procedure: exhibit register, sealed and labelled packaging, signed handovers.</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>B — Needs a named, qualified person</t>
+        </is>
+      </c>
       <c r="F19" s="19" t="n"/>
+      <c r="G19" s="20" t="n"/>
     </row>
     <row r="20" ht="34" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>02.6</t>
+          <t>02.7</t>
         </is>
       </c>
       <c r="B20" s="15" t="n"/>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>Evidence handling &amp; chain of custody</t>
+          <t>Expert witness testimony</t>
         </is>
       </c>
       <c r="D20" s="17" t="inlineStr">
         <is>
-          <t>We operate a documented chain-of-custody procedure: exhibit register, sealed and labelled packaging, signed handovers.</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="n"/>
+          <t>We have someone who could realistically be accepted by a court as an expert in their field and testify.</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>B — Needs a named, qualified person</t>
+        </is>
+      </c>
       <c r="F20" s="19" t="n"/>
+      <c r="G20" s="20" t="n"/>
     </row>
     <row r="21" ht="34" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>02.7</t>
+          <t>02.8</t>
         </is>
       </c>
       <c r="B21" s="15" t="n"/>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>Expert witness testimony</t>
+          <t>Court-ready forensic reporting</t>
         </is>
       </c>
       <c r="D21" s="17" t="inlineStr">
         <is>
-          <t>We have someone who could realistically be accepted by a court as an expert in their field and testify.</t>
-        </is>
-      </c>
-      <c r="E21" s="18" t="n"/>
+          <t>We produce reports written to a standard suitable for court, a CCMA matter or a disciplinary hearing.</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>B — Needs a named, qualified person</t>
+        </is>
+      </c>
       <c r="F21" s="19" t="n"/>
-    </row>
-    <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>02.8</t>
-        </is>
-      </c>
-      <c r="B22" s="15" t="n"/>
-      <c r="C22" s="16" t="inlineStr">
-        <is>
-          <t>Court-ready forensic reporting</t>
-        </is>
-      </c>
-      <c r="D22" s="17" t="inlineStr">
-        <is>
-          <t>We produce reports written to a standard suitable for court, a CCMA matter or a disciplinary hearing.</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="n"/>
-      <c r="F22" s="19" t="n"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="G21" s="20" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Polygraph Services</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>8 services</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="n"/>
-      <c r="E23" s="13" t="n"/>
-      <c r="F23" s="13" t="n"/>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>5 parked</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="n"/>
+      <c r="E22" s="13" t="n"/>
+      <c r="F22" s="13" t="n"/>
+      <c r="G22" s="13" t="n"/>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>03.1</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Periodic integrity testing</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>We can run scheduled, repeat integrity examinations for a client's staff.</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>C — Plausible extension of confirmed work</t>
+        </is>
+      </c>
+      <c r="F23" s="19" t="n"/>
+      <c r="G23" s="20" t="n"/>
     </row>
     <row r="24" ht="34" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>03.1</t>
+          <t>03.2</t>
         </is>
       </c>
       <c r="B24" s="15" t="n"/>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>Pre-employment screening examinations</t>
+          <t>Theft &amp; shrinkage investigations</t>
         </is>
       </c>
       <c r="D24" s="17" t="inlineStr">
         <is>
-          <t>We have a trained polygraph examiner and working instrumentation available for pre-employment screening.</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="n"/>
+          <t>We use polygraph examinations as one input in theft and stock-loss investigations.</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>C — Plausible extension of confirmed work</t>
+        </is>
+      </c>
       <c r="F24" s="19" t="n"/>
+      <c r="G24" s="20" t="n"/>
     </row>
     <row r="25" ht="34" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>03.2</t>
+          <t>03.3</t>
         </is>
       </c>
       <c r="B25" s="15" t="n"/>
       <c r="C25" s="16" t="inlineStr">
         <is>
-          <t>Periodic integrity testing</t>
+          <t>Internal integrity programmes</t>
         </is>
       </c>
       <c r="D25" s="17" t="inlineStr">
         <is>
-          <t>We can run scheduled, repeat integrity examinations for a client's staff.</t>
-        </is>
-      </c>
-      <c r="E25" s="18" t="n"/>
+          <t>We can design and run an ongoing integrity-testing programme for a client.</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>C — Plausible extension of confirmed work</t>
+        </is>
+      </c>
       <c r="F25" s="19" t="n"/>
+      <c r="G25" s="20" t="n"/>
     </row>
     <row r="26" ht="34" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>03.3</t>
+          <t>03.4</t>
         </is>
       </c>
       <c r="B26" s="15" t="n"/>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>Specific-issue (incident) examinations</t>
+          <t>Structured pre-test interviewing</t>
         </is>
       </c>
       <c r="D26" s="17" t="inlineStr">
         <is>
-          <t>We run single-issue examinations tied to a specific incident.</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="n"/>
+          <t>Every examination includes a structured pre-test interview and written informed consent.</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>D — Superseded or narrow</t>
+        </is>
+      </c>
       <c r="F26" s="19" t="n"/>
+      <c r="G26" s="20" t="n"/>
     </row>
     <row r="27" ht="34" customHeight="1">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>03.4</t>
+          <t>03.5</t>
         </is>
       </c>
       <c r="B27" s="15" t="n"/>
       <c r="C27" s="16" t="inlineStr">
         <is>
-          <t>Theft &amp; shrinkage investigations</t>
+          <t>Documented examination reporting</t>
         </is>
       </c>
       <c r="D27" s="17" t="inlineStr">
         <is>
-          <t>We use polygraph examinations as one input in theft and stock-loss investigations.</t>
-        </is>
-      </c>
-      <c r="E27" s="18" t="n"/>
+          <t>Every examination produces a written report recording the questions, the data and the examiner's opinion.</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>D — Superseded or narrow</t>
+        </is>
+      </c>
       <c r="F27" s="19" t="n"/>
-    </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="14" t="inlineStr">
-        <is>
-          <t>03.5</t>
-        </is>
-      </c>
-      <c r="B28" s="15" t="n"/>
-      <c r="C28" s="16" t="inlineStr">
-        <is>
-          <t>Disciplinary hearing support</t>
-        </is>
-      </c>
-      <c r="D28" s="17" t="inlineStr">
-        <is>
-          <t>We provide examination reports for use in an employer's disciplinary process, as supporting material rather than proof.</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="n"/>
-      <c r="F28" s="19" t="n"/>
+      <c r="G27" s="20" t="n"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Security Services</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>7 parked</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="n"/>
+      <c r="E28" s="13" t="n"/>
+      <c r="F28" s="13" t="n"/>
+      <c r="G28" s="13" t="n"/>
     </row>
     <row r="29" ht="34" customHeight="1">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>03.6</t>
+          <t>04.1</t>
         </is>
       </c>
       <c r="B29" s="15" t="n"/>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>Internal integrity programmes</t>
+          <t>Access control &amp; visitor management</t>
         </is>
       </c>
       <c r="D29" s="17" t="inlineStr">
         <is>
-          <t>We can design and run an ongoing integrity-testing programme for a client.</t>
-        </is>
-      </c>
-      <c r="E29" s="18" t="n"/>
+          <t>We can design and implement access-control and visitor-management systems.</t>
+        </is>
+      </c>
+      <c r="E29" s="18" t="inlineStr">
+        <is>
+          <t>A — Significant capability absent from your profile</t>
+        </is>
+      </c>
       <c r="F29" s="19" t="n"/>
+      <c r="G29" s="20" t="n"/>
     </row>
     <row r="30" ht="34" customHeight="1">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>03.7</t>
+          <t>04.2</t>
         </is>
       </c>
       <c r="B30" s="15" t="n"/>
       <c r="C30" s="16" t="inlineStr">
         <is>
-          <t>Structured pre-test interviewing</t>
+          <t>CCTV design, installation &amp; monitoring</t>
         </is>
       </c>
       <c r="D30" s="17" t="inlineStr">
         <is>
-          <t>Every examination includes a structured pre-test interview and written informed consent.</t>
-        </is>
-      </c>
-      <c r="E30" s="18" t="n"/>
+          <t>We can specify, physically install and monitor CCTV. If we only advise or only monitor, mark this FALSE and say which.</t>
+        </is>
+      </c>
+      <c r="E30" s="18" t="inlineStr">
+        <is>
+          <t>A — Significant capability absent from your profile</t>
+        </is>
+      </c>
       <c r="F30" s="19" t="n"/>
+      <c r="G30" s="20" t="n"/>
     </row>
     <row r="31" ht="34" customHeight="1">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>03.8</t>
+          <t>04.3</t>
         </is>
       </c>
       <c r="B31" s="15" t="n"/>
       <c r="C31" s="16" t="inlineStr">
         <is>
-          <t>Documented examination reporting</t>
+          <t>Alarm systems &amp; response coordination</t>
         </is>
       </c>
       <c r="D31" s="17" t="inlineStr">
         <is>
-          <t>Every examination produces a written report recording the questions, the data and the examiner's opinion.</t>
-        </is>
-      </c>
-      <c r="E31" s="18" t="n"/>
+          <t>We can install or specify alarm systems and coordinate an armed-response arrangement.</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="inlineStr">
+        <is>
+          <t>A — Significant capability absent from your profile</t>
+        </is>
+      </c>
       <c r="F31" s="19" t="n"/>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>Security Services</t>
-        </is>
-      </c>
-      <c r="C32" s="12" t="inlineStr">
-        <is>
-          <t>8 services</t>
-        </is>
-      </c>
-      <c r="D32" s="13" t="n"/>
-      <c r="E32" s="13" t="n"/>
-      <c r="F32" s="13" t="n"/>
+      <c r="G31" s="20" t="n"/>
+    </row>
+    <row r="32" ht="34" customHeight="1">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>04.4</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="n"/>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>Perimeter &amp; physical security design</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>We can design perimeter and physical security measures — fencing, lighting, barriers, layout.</t>
+        </is>
+      </c>
+      <c r="E32" s="18" t="inlineStr">
+        <is>
+          <t>A — Significant capability absent from your profile</t>
+        </is>
+      </c>
+      <c r="F32" s="19" t="n"/>
+      <c r="G32" s="20" t="n"/>
     </row>
     <row r="33" ht="34" customHeight="1">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>04.1</t>
+          <t>04.5</t>
         </is>
       </c>
       <c r="B33" s="15" t="n"/>
       <c r="C33" s="16" t="inlineStr">
         <is>
-          <t>Security risk assessments</t>
+          <t>Control room &amp; monitoring solutions</t>
         </is>
       </c>
       <c r="D33" s="17" t="inlineStr">
         <is>
-          <t>We can survey a site or an operation and produce a written risk assessment with recommendations.</t>
-        </is>
-      </c>
-      <c r="E33" s="18" t="n"/>
+          <t>We can set up or supply a control room / monitoring capability.</t>
+        </is>
+      </c>
+      <c r="E33" s="18" t="inlineStr">
+        <is>
+          <t>A — Significant capability absent from your profile</t>
+        </is>
+      </c>
       <c r="F33" s="19" t="n"/>
+      <c r="G33" s="20" t="n"/>
     </row>
     <row r="34" ht="34" customHeight="1">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>04.2</t>
+          <t>04.6</t>
         </is>
       </c>
       <c r="B34" s="15" t="n"/>
       <c r="C34" s="16" t="inlineStr">
         <is>
-          <t>Access control &amp; visitor management</t>
+          <t>Security policy &amp; SOP development</t>
         </is>
       </c>
       <c r="D34" s="17" t="inlineStr">
         <is>
-          <t>We can design and implement access-control and visitor-management systems.</t>
-        </is>
-      </c>
-      <c r="E34" s="18" t="n"/>
+          <t>We write security policies, post orders and standard operating procedures for clients.</t>
+        </is>
+      </c>
+      <c r="E34" s="18" t="inlineStr">
+        <is>
+          <t>C — Plausible extension of confirmed work</t>
+        </is>
+      </c>
       <c r="F34" s="19" t="n"/>
+      <c r="G34" s="20" t="n"/>
     </row>
     <row r="35" ht="34" customHeight="1">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>04.3</t>
+          <t>04.7</t>
         </is>
       </c>
       <c r="B35" s="15" t="n"/>
       <c r="C35" s="16" t="inlineStr">
         <is>
-          <t>CCTV design, installation &amp; monitoring</t>
+          <t>Security audits &amp; compliance reviews</t>
         </is>
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>We can specify, physically install and monitor CCTV. If we only advise or only monitor, mark this FALSE and say which.</t>
-        </is>
-      </c>
-      <c r="E35" s="18" t="n"/>
+          <t>We audit an existing security setup against its own policies or applicable requirements.</t>
+        </is>
+      </c>
+      <c r="E35" s="18" t="inlineStr">
+        <is>
+          <t>C — Plausible extension of confirmed work</t>
+        </is>
+      </c>
       <c r="F35" s="19" t="n"/>
-    </row>
-    <row r="36" ht="34" customHeight="1">
-      <c r="A36" s="14" t="inlineStr">
-        <is>
-          <t>04.4</t>
-        </is>
-      </c>
-      <c r="B36" s="15" t="n"/>
-      <c r="C36" s="16" t="inlineStr">
-        <is>
-          <t>Alarm systems &amp; response coordination</t>
-        </is>
-      </c>
-      <c r="D36" s="17" t="inlineStr">
-        <is>
-          <t>We can install or specify alarm systems and coordinate an armed-response arrangement.</t>
-        </is>
-      </c>
-      <c r="E36" s="18" t="n"/>
-      <c r="F36" s="19" t="n"/>
+      <c r="G35" s="20" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Protection Services</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>4 parked</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="n"/>
+      <c r="E36" s="13" t="n"/>
+      <c r="F36" s="13" t="n"/>
+      <c r="G36" s="13" t="n"/>
     </row>
     <row r="37" ht="34" customHeight="1">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>04.5</t>
+          <t>05.1</t>
         </is>
       </c>
       <c r="B37" s="15" t="n"/>
       <c r="C37" s="16" t="inlineStr">
         <is>
-          <t>Perimeter &amp; physical security design</t>
+          <t>Family &amp; residential protection</t>
         </is>
       </c>
       <c r="D37" s="17" t="inlineStr">
         <is>
-          <t>We can design perimeter and physical security measures — fencing, lighting, barriers, layout.</t>
-        </is>
-      </c>
-      <c r="E37" s="18" t="n"/>
+          <t>We provide protection covering a principal's family and residence.</t>
+        </is>
+      </c>
+      <c r="E37" s="18" t="inlineStr">
+        <is>
+          <t>C — Plausible extension of confirmed work</t>
+        </is>
+      </c>
       <c r="F37" s="19" t="n"/>
+      <c r="G37" s="20" t="n"/>
     </row>
     <row r="38" ht="34" customHeight="1">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>04.6</t>
+          <t>05.2</t>
         </is>
       </c>
       <c r="B38" s="15" t="n"/>
       <c r="C38" s="16" t="inlineStr">
         <is>
-          <t>Control room &amp; monitoring solutions</t>
+          <t>Travel risk management &amp; advance work</t>
         </is>
       </c>
       <c r="D38" s="17" t="inlineStr">
         <is>
-          <t>We can set up or supply a control room / monitoring capability.</t>
-        </is>
-      </c>
-      <c r="E38" s="18" t="n"/>
+          <t>We conduct route planning, venue advance work and travel risk assessment before a movement.</t>
+        </is>
+      </c>
+      <c r="E38" s="18" t="inlineStr">
+        <is>
+          <t>C — Plausible extension of confirmed work</t>
+        </is>
+      </c>
       <c r="F38" s="19" t="n"/>
+      <c r="G38" s="20" t="n"/>
     </row>
     <row r="39" ht="34" customHeight="1">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>04.7</t>
+          <t>05.3</t>
         </is>
       </c>
       <c r="B39" s="15" t="n"/>
       <c r="C39" s="16" t="inlineStr">
         <is>
-          <t>Security policy &amp; SOP development</t>
+          <t>Threat &amp; vulnerability assessment</t>
         </is>
       </c>
       <c r="D39" s="17" t="inlineStr">
         <is>
-          <t>We write security policies, post orders and standard operating procedures for clients.</t>
-        </is>
-      </c>
-      <c r="E39" s="18" t="n"/>
+          <t>We assess threats against an individual and produce a written protective assessment.</t>
+        </is>
+      </c>
+      <c r="E39" s="18" t="inlineStr">
+        <is>
+          <t>C — Plausible extension of confirmed work</t>
+        </is>
+      </c>
       <c r="F39" s="19" t="n"/>
+      <c r="G39" s="20" t="n"/>
     </row>
     <row r="40" ht="34" customHeight="1">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>04.8</t>
+          <t>05.4</t>
         </is>
       </c>
       <c r="B40" s="15" t="n"/>
       <c r="C40" s="16" t="inlineStr">
         <is>
-          <t>Security audits &amp; compliance reviews</t>
+          <t>Female close protection officers</t>
         </is>
       </c>
       <c r="D40" s="17" t="inlineStr">
         <is>
-          <t>We audit an existing security setup against its own policies or applicable requirements.</t>
-        </is>
-      </c>
-      <c r="E40" s="18" t="n"/>
+          <t>We have at least one female close protection officer on the team or reliably available.</t>
+        </is>
+      </c>
+      <c r="E40" s="18" t="inlineStr">
+        <is>
+          <t>D — Superseded or narrow</t>
+        </is>
+      </c>
       <c r="F40" s="19" t="n"/>
+      <c r="G40" s="20" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>Protection Services</t>
+          <t>Guarding Services</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>8 services</t>
+          <t>8 parked</t>
         </is>
       </c>
       <c r="D41" s="13" t="n"/>
       <c r="E41" s="13" t="n"/>
       <c r="F41" s="13" t="n"/>
+      <c r="G41" s="13" t="n"/>
     </row>
     <row r="42" ht="34" customHeight="1">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>05.1</t>
+          <t>06.1</t>
         </is>
       </c>
       <c r="B42" s="15" t="n"/>
       <c r="C42" s="16" t="inlineStr">
         <is>
-          <t>Close protection officers</t>
+          <t>Static &amp; site guarding</t>
         </is>
       </c>
       <c r="D42" s="17" t="inlineStr">
         <is>
-          <t>We have PSIRA-registered close protection officers, graded for the role, available for deployment.</t>
-        </is>
-      </c>
-      <c r="E42" s="18" t="n"/>
+          <t>We deploy PSIRA-registered guards to static posts and sites.</t>
+        </is>
+      </c>
+      <c r="E42" s="18" t="inlineStr">
+        <is>
+          <t>A — Significant capability absent from your profile</t>
+        </is>
+      </c>
       <c r="F42" s="19" t="n"/>
+      <c r="G42" s="20" t="n"/>
     </row>
     <row r="43" ht="34" customHeight="1">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>05.2</t>
+          <t>06.2</t>
         </is>
       </c>
       <c r="B43" s="15" t="n"/>
       <c r="C43" s="16" t="inlineStr">
         <is>
-          <t>Executive &amp; corporate protection</t>
+          <t>Access control officers</t>
         </is>
       </c>
       <c r="D43" s="17" t="inlineStr">
         <is>
-          <t>We provide protection details for company executives and corporate clients.</t>
-        </is>
-      </c>
-      <c r="E43" s="18" t="n"/>
+          <t>We supply officers specifically for gate and access-control duty.</t>
+        </is>
+      </c>
+      <c r="E43" s="18" t="inlineStr">
+        <is>
+          <t>C — Plausible extension of confirmed work</t>
+        </is>
+      </c>
       <c r="F43" s="19" t="n"/>
+      <c r="G43" s="20" t="n"/>
     </row>
     <row r="44" ht="34" customHeight="1">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>05.3</t>
+          <t>06.3</t>
         </is>
       </c>
       <c r="B44" s="15" t="n"/>
       <c r="C44" s="16" t="inlineStr">
         <is>
-          <t>Family &amp; residential protection</t>
+          <t>Residential estate guarding</t>
         </is>
       </c>
       <c r="D44" s="17" t="inlineStr">
         <is>
-          <t>We provide protection covering a principal's family and residence.</t>
-        </is>
-      </c>
-      <c r="E44" s="18" t="n"/>
+          <t>We guard residential estates and complexes.</t>
+        </is>
+      </c>
+      <c r="E44" s="18" t="inlineStr">
+        <is>
+          <t>A — Significant capability absent from your profile</t>
+        </is>
+      </c>
       <c r="F44" s="19" t="n"/>
+      <c r="G44" s="20" t="n"/>
     </row>
     <row r="45" ht="34" customHeight="1">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>05.4</t>
+          <t>06.4</t>
         </is>
       </c>
       <c r="B45" s="15" t="n"/>
       <c r="C45" s="16" t="inlineStr">
         <is>
-          <t>Secure chauffeur &amp; transport</t>
+          <t>Retail &amp; commercial guarding</t>
         </is>
       </c>
       <c r="D45" s="17" t="inlineStr">
         <is>
-          <t>We can provide trained security drivers and secure transport.</t>
-        </is>
-      </c>
-      <c r="E45" s="18" t="n"/>
+          <t>We guard retail and commercial premises.</t>
+        </is>
+      </c>
+      <c r="E45" s="18" t="inlineStr">
+        <is>
+          <t>A — Significant capability absent from your profile</t>
+        </is>
+      </c>
       <c r="F45" s="19" t="n"/>
+      <c r="G45" s="20" t="n"/>
     </row>
     <row r="46" ht="34" customHeight="1">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>05.5</t>
+          <t>06.5</t>
         </is>
       </c>
       <c r="B46" s="15" t="n"/>
       <c r="C46" s="16" t="inlineStr">
         <is>
-          <t>Travel risk management &amp; advance work</t>
+          <t>Construction &amp; industrial site security</t>
         </is>
       </c>
       <c r="D46" s="17" t="inlineStr">
         <is>
-          <t>We conduct route planning, venue advance work and travel risk assessment before a movement.</t>
-        </is>
-      </c>
-      <c r="E46" s="18" t="n"/>
+          <t>We secure construction sites and industrial premises.</t>
+        </is>
+      </c>
+      <c r="E46" s="18" t="inlineStr">
+        <is>
+          <t>A — Significant capability absent from your profile</t>
+        </is>
+      </c>
       <c r="F46" s="19" t="n"/>
+      <c r="G46" s="20" t="n"/>
     </row>
     <row r="47" ht="34" customHeight="1">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>05.6</t>
+          <t>06.6</t>
         </is>
       </c>
       <c r="B47" s="15" t="n"/>
       <c r="C47" s="16" t="inlineStr">
         <is>
-          <t>Event &amp; dignitary protection</t>
+          <t>Mobile patrols &amp; guard monitoring</t>
         </is>
       </c>
       <c r="D47" s="17" t="inlineStr">
         <is>
-          <t>We provide protection at events and for visiting dignitaries.</t>
-        </is>
-      </c>
-      <c r="E47" s="18" t="n"/>
+          <t>We run mobile patrols and monitor guards on shift, with a record of visits or checkpoints.</t>
+        </is>
+      </c>
+      <c r="E47" s="18" t="inlineStr">
+        <is>
+          <t>A — Significant capability absent from your profile</t>
+        </is>
+      </c>
       <c r="F47" s="19" t="n"/>
+      <c r="G47" s="20" t="n"/>
     </row>
     <row r="48" ht="34" customHeight="1">
       <c r="A48" s="14" t="inlineStr">
         <is>
-          <t>05.7</t>
+          <t>06.7</t>
         </is>
       </c>
       <c r="B48" s="15" t="n"/>
       <c r="C48" s="16" t="inlineStr">
         <is>
-          <t>Threat &amp; vulnerability assessment</t>
+          <t>Reaction &amp; response officers</t>
         </is>
       </c>
       <c r="D48" s="17" t="inlineStr">
         <is>
-          <t>We assess threats against an individual and produce a written protective assessment.</t>
-        </is>
-      </c>
-      <c r="E48" s="18" t="n"/>
+          <t>We field reaction or response officers, whether our own or through a formal arrangement.</t>
+        </is>
+      </c>
+      <c r="E48" s="18" t="inlineStr">
+        <is>
+          <t>A — Significant capability absent from your profile</t>
+        </is>
+      </c>
       <c r="F48" s="19" t="n"/>
+      <c r="G48" s="20" t="n"/>
     </row>
     <row r="49" ht="34" customHeight="1">
       <c r="A49" s="14" t="inlineStr">
         <is>
-          <t>05.8</t>
+          <t>06.8</t>
         </is>
       </c>
       <c r="B49" s="15" t="n"/>
       <c r="C49" s="16" t="inlineStr">
         <is>
-          <t>Female close protection officers</t>
+          <t>Supervision &amp; control room staffing</t>
         </is>
       </c>
       <c r="D49" s="17" t="inlineStr">
         <is>
-          <t>We have at least one female close protection officer on the team or reliably available.</t>
-        </is>
-      </c>
-      <c r="E49" s="18" t="n"/>
+          <t>We supply supervisors and control-room operators, not only guards.</t>
+        </is>
+      </c>
+      <c r="E49" s="18" t="inlineStr">
+        <is>
+          <t>D — Superseded or narrow</t>
+        </is>
+      </c>
       <c r="F49" s="19" t="n"/>
+      <c r="G49" s="20" t="n"/>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="10" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>Guarding Services</t>
+          <t>Specialized Services</t>
         </is>
       </c>
       <c r="C50" s="12" t="inlineStr">
         <is>
-          <t>8 services</t>
+          <t>5 parked</t>
         </is>
       </c>
       <c r="D50" s="13" t="n"/>
       <c r="E50" s="13" t="n"/>
       <c r="F50" s="13" t="n"/>
+      <c r="G50" s="13" t="n"/>
     </row>
     <row r="51" ht="34" customHeight="1">
       <c r="A51" s="14" t="inlineStr">
         <is>
-          <t>06.1</t>
+          <t>07.1</t>
         </is>
       </c>
       <c r="B51" s="15" t="n"/>
       <c r="C51" s="16" t="inlineStr">
         <is>
-          <t>Static &amp; site guarding</t>
+          <t>Tactical &amp; refresher training</t>
         </is>
       </c>
       <c r="D51" s="17" t="inlineStr">
         <is>
-          <t>We deploy PSIRA-registered guards to static posts and sites.</t>
-        </is>
-      </c>
-      <c r="E51" s="18" t="n"/>
+          <t>We run tactical and refresher shooting or handling courses beyond basic competency.</t>
+        </is>
+      </c>
+      <c r="E51" s="18" t="inlineStr">
+        <is>
+          <t>D — Superseded or narrow</t>
+        </is>
+      </c>
       <c r="F51" s="19" t="n"/>
+      <c r="G51" s="20" t="n"/>
     </row>
     <row r="52" ht="34" customHeight="1">
       <c r="A52" s="14" t="inlineStr">
         <is>
-          <t>06.2</t>
+          <t>07.2</t>
         </is>
       </c>
       <c r="B52" s="15" t="n"/>
       <c r="C52" s="16" t="inlineStr">
         <is>
-          <t>Access control officers</t>
+          <t>Valuable goods &amp; cash escorts</t>
         </is>
       </c>
       <c r="D52" s="17" t="inlineStr">
         <is>
-          <t>We supply officers specifically for gate and access-control duty.</t>
-        </is>
-      </c>
-      <c r="E52" s="18" t="n"/>
+          <t>We escort valuable goods or cash. Note: cash-in-transit is separately regulated — confirm we are permitted for what we advertise.</t>
+        </is>
+      </c>
+      <c r="E52" s="18" t="inlineStr">
+        <is>
+          <t>D — Superseded or narrow</t>
+        </is>
+      </c>
       <c r="F52" s="19" t="n"/>
+      <c r="G52" s="20" t="n"/>
     </row>
     <row r="53" ht="34" customHeight="1">
       <c r="A53" s="14" t="inlineStr">
         <is>
-          <t>06.3</t>
+          <t>07.3</t>
         </is>
       </c>
       <c r="B53" s="15" t="n"/>
       <c r="C53" s="16" t="inlineStr">
         <is>
-          <t>Residential estate guarding</t>
+          <t>Asset &amp; vehicle recovery</t>
         </is>
       </c>
       <c r="D53" s="17" t="inlineStr">
         <is>
-          <t>We guard residential estates and complexes.</t>
-        </is>
-      </c>
-      <c r="E53" s="18" t="n"/>
+          <t>We trace and recover stolen assets and vehicles, lawfully and with SAPS involvement where required.</t>
+        </is>
+      </c>
+      <c r="E53" s="18" t="inlineStr">
+        <is>
+          <t>D — Superseded or narrow</t>
+        </is>
+      </c>
       <c r="F53" s="19" t="n"/>
+      <c r="G53" s="20" t="n"/>
     </row>
     <row r="54" ht="34" customHeight="1">
       <c r="A54" s="14" t="inlineStr">
         <is>
-          <t>06.4</t>
+          <t>07.4</t>
         </is>
       </c>
       <c r="B54" s="15" t="n"/>
       <c r="C54" s="16" t="inlineStr">
         <is>
-          <t>Retail &amp; commercial guarding</t>
+          <t>Loss prevention programmes</t>
         </is>
       </c>
       <c r="D54" s="17" t="inlineStr">
         <is>
-          <t>We guard retail and commercial premises.</t>
-        </is>
-      </c>
-      <c r="E54" s="18" t="n"/>
+          <t>We design and run ongoing loss-prevention programmes for clients.</t>
+        </is>
+      </c>
+      <c r="E54" s="18" t="inlineStr">
+        <is>
+          <t>D — Superseded or narrow</t>
+        </is>
+      </c>
       <c r="F54" s="19" t="n"/>
+      <c r="G54" s="20" t="n"/>
     </row>
     <row r="55" ht="34" customHeight="1">
       <c r="A55" s="14" t="inlineStr">
         <is>
-          <t>06.5</t>
+          <t>07.5</t>
         </is>
       </c>
       <c r="B55" s="15" t="n"/>
       <c r="C55" s="16" t="inlineStr">
         <is>
-          <t>Construction &amp; industrial site security</t>
+          <t>Undercover operative placement</t>
         </is>
       </c>
       <c r="D55" s="17" t="inlineStr">
         <is>
-          <t>We secure construction sites and industrial premises.</t>
-        </is>
-      </c>
-      <c r="E55" s="18" t="n"/>
+          <t>We place undercover operatives inside a client's workplace, with a lawful basis and the client's written mandate.</t>
+        </is>
+      </c>
+      <c r="E55" s="18" t="inlineStr">
+        <is>
+          <t>D — Superseded or narrow</t>
+        </is>
+      </c>
       <c r="F55" s="19" t="n"/>
-    </row>
-    <row r="56" ht="34" customHeight="1">
-      <c r="A56" s="14" t="inlineStr">
-        <is>
-          <t>06.6</t>
-        </is>
-      </c>
-      <c r="B56" s="15" t="n"/>
-      <c r="C56" s="16" t="inlineStr">
-        <is>
-          <t>Mobile patrols &amp; guard monitoring</t>
-        </is>
-      </c>
-      <c r="D56" s="17" t="inlineStr">
-        <is>
-          <t>We run mobile patrols and monitor guards on shift, with a record of visits or checkpoints.</t>
-        </is>
-      </c>
-      <c r="E56" s="18" t="n"/>
-      <c r="F56" s="19" t="n"/>
-    </row>
-    <row r="57" ht="34" customHeight="1">
-      <c r="A57" s="14" t="inlineStr">
-        <is>
-          <t>06.7</t>
-        </is>
-      </c>
-      <c r="B57" s="15" t="n"/>
-      <c r="C57" s="16" t="inlineStr">
-        <is>
-          <t>Reaction &amp; response officers</t>
-        </is>
-      </c>
-      <c r="D57" s="17" t="inlineStr">
-        <is>
-          <t>We field reaction or response officers, whether our own or through a formal arrangement.</t>
-        </is>
-      </c>
-      <c r="E57" s="18" t="n"/>
-      <c r="F57" s="19" t="n"/>
-    </row>
-    <row r="58" ht="34" customHeight="1">
-      <c r="A58" s="14" t="inlineStr">
-        <is>
-          <t>06.8</t>
-        </is>
-      </c>
-      <c r="B58" s="15" t="n"/>
-      <c r="C58" s="16" t="inlineStr">
-        <is>
-          <t>Supervision &amp; control room staffing</t>
-        </is>
-      </c>
-      <c r="D58" s="17" t="inlineStr">
-        <is>
-          <t>We supply supervisors and control-room operators, not only guards.</t>
-        </is>
-      </c>
-      <c r="E58" s="18" t="n"/>
-      <c r="F58" s="19" t="n"/>
-    </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="10" t="inlineStr">
-        <is>
-          <t>07</t>
-        </is>
-      </c>
-      <c r="B59" s="11" t="inlineStr">
-        <is>
-          <t>Specialized Services</t>
-        </is>
-      </c>
-      <c r="C59" s="12" t="inlineStr">
-        <is>
-          <t>8 services</t>
-        </is>
-      </c>
-      <c r="D59" s="13" t="n"/>
-      <c r="E59" s="13" t="n"/>
-      <c r="F59" s="13" t="n"/>
-    </row>
-    <row r="60" ht="34" customHeight="1">
-      <c r="A60" s="14" t="inlineStr">
-        <is>
-          <t>07.1</t>
-        </is>
-      </c>
-      <c r="B60" s="15" t="n"/>
-      <c r="C60" s="16" t="inlineStr">
-        <is>
-          <t>Accredited firearm training</t>
-        </is>
-      </c>
-      <c r="D60" s="17" t="inlineStr">
-        <is>
-          <t>We hold current accreditation to deliver firearm competency training, or deliver it through an accredited partner.</t>
-        </is>
-      </c>
-      <c r="E60" s="18" t="n"/>
-      <c r="F60" s="19" t="n"/>
-    </row>
-    <row r="61" ht="34" customHeight="1">
-      <c r="A61" s="14" t="inlineStr">
-        <is>
-          <t>07.2</t>
-        </is>
-      </c>
-      <c r="B61" s="15" t="n"/>
-      <c r="C61" s="16" t="inlineStr">
-        <is>
-          <t>Tactical &amp; refresher training</t>
-        </is>
-      </c>
-      <c r="D61" s="17" t="inlineStr">
-        <is>
-          <t>We run tactical and refresher shooting or handling courses beyond basic competency.</t>
-        </is>
-      </c>
-      <c r="E61" s="18" t="n"/>
-      <c r="F61" s="19" t="n"/>
-    </row>
-    <row r="62" ht="34" customHeight="1">
-      <c r="A62" s="14" t="inlineStr">
-        <is>
-          <t>07.3</t>
-        </is>
-      </c>
-      <c r="B62" s="15" t="n"/>
-      <c r="C62" s="16" t="inlineStr">
-        <is>
-          <t>Valuable goods &amp; cash escorts</t>
-        </is>
-      </c>
-      <c r="D62" s="17" t="inlineStr">
-        <is>
-          <t>We escort valuable goods or cash. Note: cash-in-transit is separately regulated — confirm we are permitted for what we advertise.</t>
-        </is>
-      </c>
-      <c r="E62" s="18" t="n"/>
-      <c r="F62" s="19" t="n"/>
-    </row>
-    <row r="63" ht="34" customHeight="1">
-      <c r="A63" s="14" t="inlineStr">
-        <is>
-          <t>07.4</t>
-        </is>
-      </c>
-      <c r="B63" s="15" t="n"/>
-      <c r="C63" s="16" t="inlineStr">
-        <is>
-          <t>Asset &amp; vehicle recovery</t>
-        </is>
-      </c>
-      <c r="D63" s="17" t="inlineStr">
-        <is>
-          <t>We trace and recover stolen assets and vehicles, lawfully and with SAPS involvement where required.</t>
-        </is>
-      </c>
-      <c r="E63" s="18" t="n"/>
-      <c r="F63" s="19" t="n"/>
-    </row>
-    <row r="64" ht="34" customHeight="1">
-      <c r="A64" s="14" t="inlineStr">
-        <is>
-          <t>07.5</t>
-        </is>
-      </c>
-      <c r="B64" s="15" t="n"/>
-      <c r="C64" s="16" t="inlineStr">
-        <is>
-          <t>Loss prevention programmes</t>
-        </is>
-      </c>
-      <c r="D64" s="17" t="inlineStr">
-        <is>
-          <t>We design and run ongoing loss-prevention programmes for clients.</t>
-        </is>
-      </c>
-      <c r="E64" s="18" t="n"/>
-      <c r="F64" s="19" t="n"/>
-    </row>
-    <row r="65" ht="34" customHeight="1">
-      <c r="A65" s="14" t="inlineStr">
-        <is>
-          <t>07.6</t>
-        </is>
-      </c>
-      <c r="B65" s="15" t="n"/>
-      <c r="C65" s="16" t="inlineStr">
-        <is>
-          <t>Undercover operative placement</t>
-        </is>
-      </c>
-      <c r="D65" s="17" t="inlineStr">
-        <is>
-          <t>We place undercover operatives inside a client's workplace, with a lawful basis and the client's written mandate.</t>
-        </is>
-      </c>
-      <c r="E65" s="18" t="n"/>
-      <c r="F65" s="19" t="n"/>
-    </row>
-    <row r="66" ht="34" customHeight="1">
-      <c r="A66" s="14" t="inlineStr">
-        <is>
-          <t>07.7</t>
-        </is>
-      </c>
-      <c r="B66" s="15" t="n"/>
-      <c r="C66" s="16" t="inlineStr">
-        <is>
-          <t>Crowd &amp; labour unrest support</t>
-        </is>
-      </c>
-      <c r="D66" s="17" t="inlineStr">
-        <is>
-          <t>We provide lawful, defensive, de-escalation-first support to a client's site during unrest. This is NOT strike-breaking.</t>
-        </is>
-      </c>
-      <c r="E66" s="18" t="n"/>
-      <c r="F66" s="19" t="n"/>
-    </row>
-    <row r="67" ht="34" customHeight="1">
-      <c r="A67" s="14" t="inlineStr">
-        <is>
-          <t>07.8</t>
-        </is>
-      </c>
-      <c r="B67" s="15" t="n"/>
-      <c r="C67" s="16" t="inlineStr">
-        <is>
-          <t>Bespoke risk solutions</t>
-        </is>
-      </c>
-      <c r="D67" s="17" t="inlineStr">
-        <is>
-          <t>We take on bespoke briefs that fall outside the standard categories.</t>
-        </is>
-      </c>
-      <c r="E67" s="18" t="n"/>
-      <c r="F67" s="19" t="n"/>
-    </row>
-    <row r="69">
-      <c r="C69" s="5" t="inlineStr">
+      <c r="G55" s="20" t="n"/>
+    </row>
+    <row r="57">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>Progress</t>
         </is>
       </c>
-      <c r="D69" s="3" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>Answered</t>
         </is>
       </c>
-      <c r="E69" s="3">
-        <f>COUNTIF(E5:E67,"TRUE")+COUNTIF(E5:E67,"FALSE")+COUNTIF(E5:E67,"NEEDS REWORDING")</f>
+      <c r="F57" s="3">
+        <f>COUNTIF(F5:F55,"TRUE")+COUNTIF(F5:F55,"FALSE")+COUNTIF(F5:F55,"NEEDS REWORDING")</f>
         <v/>
       </c>
-      <c r="F69" s="9" t="inlineStr">
-        <is>
-          <t>of 56 services</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="D70" s="20" t="inlineStr">
-        <is>
-          <t>Marked TRUE</t>
-        </is>
-      </c>
-      <c r="E70" s="20">
-        <f>COUNTIF(E5:E67,"TRUE")</f>
+      <c r="G57" s="9" t="inlineStr">
+        <is>
+          <t>of 44 parked services</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="D58" s="21" t="inlineStr">
+        <is>
+          <t>TRUE — we will put these back</t>
+        </is>
+      </c>
+      <c r="F58" s="21">
+        <f>COUNTIF(F5:F55,"TRUE")</f>
         <v/>
       </c>
     </row>
-    <row r="71">
-      <c r="D71" s="20" t="inlineStr">
-        <is>
-          <t>Marked FALSE — will be removed</t>
-        </is>
-      </c>
-      <c r="E71" s="20">
-        <f>COUNTIF(E5:E67,"FALSE")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="D72" s="20" t="inlineStr">
-        <is>
-          <t>Needs rewording</t>
-        </is>
-      </c>
-      <c r="E72" s="20">
-        <f>COUNTIF(E5:E67,"NEEDS REWORDING")</f>
+    <row r="59">
+      <c r="D59" s="21" t="inlineStr">
+        <is>
+          <t>FALSE — these stay off</t>
+        </is>
+      </c>
+      <c r="F59" s="21">
+        <f>COUNTIF(F5:F55,"FALSE")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E6 E7 E8 E9 E10 E11 E12 E13 E15 E16 E17 E18 E19 E20 E21 E22 E24 E25 E26 E27 E28 E29 E30 E31 E33 E34 E35 E36 E37 E38 E39 E40 E42 E43 E44 E45 E46 E47 E48 E49 E51 E52 E53 E54 E55 E56 E57 E58 E60 E61 E62 E63 E64 E65 E66 E67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Pick one of the options" error="Choose TRUE, FALSE or NEEDS REWORDING from the list." type="list">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F14 F15 F16 F17 F18 F19 F20 F21 F23 F24 F25 F26 F27 F29 F30 F31 F32 F33 F34 F35 F37 F38 F39 F40 F42 F43 F44 F45 F46 F47 F48 F49 F51 F52 F53 F54 F55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Pick one of the options" error="Choose TRUE, FALSE or NEEDS REWORDING from the list." type="list">
       <formula1>"TRUE,FALSE,NEEDS REWORDING"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2148,6 +2134,426 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>What your website says today</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Taken straight from your business profile. Please check nothing here is wrong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Division</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Correct?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>01 Investigation</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>7 live</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="15" t="n"/>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Track and Trace</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="15" t="n"/>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Vetting</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="15" t="n"/>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Criminal Record Checks</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="15" t="n"/>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Extortion Cases</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="15" t="n"/>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Evictions</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="15" t="n"/>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Kidnap and Ransom Cases</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="n"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="15" t="n"/>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Polygraphs</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>02 Forensic</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>1 live</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="15" t="n"/>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>No itemised list — scope defined per assignment, per your profile</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>03 Polygraph</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>3 live</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="n"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="15" t="n"/>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>Examinations supporting investigations</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Screening examinations</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="15" t="n"/>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>Internal enquiry support</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>04 Security</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>4 live</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="15" t="n"/>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Risk-based security support</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="15" t="n"/>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>Asset Protection</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="15" t="n"/>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>Bullion Runs</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="15" t="n"/>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>High Value Assets in Transit</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>05 Protection</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>4 live</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="15" t="n"/>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Executive Close Protection</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="15" t="n"/>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>Corporate Executive Close Protection</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="15" t="n"/>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>Special Event Security</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="15" t="n"/>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>Secure Drivers</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>06 Guarding</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>1 live</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="15" t="n"/>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>No itemised list — scope defined per assignment, per your profile</t>
+        </is>
+      </c>
+      <c r="C30" s="19" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>07 Specialized</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>10 live</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="15" t="n"/>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>Mining Security</t>
+        </is>
+      </c>
+      <c r="C32" s="19" t="n"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="15" t="n"/>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>Illegal Mining Prevention Teams</t>
+        </is>
+      </c>
+      <c r="C33" s="19" t="n"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="15" t="n"/>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>Riot / Civil Unrest Control</t>
+        </is>
+      </c>
+      <c r="C34" s="19" t="n"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="15" t="n"/>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>Dedicated Searches</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="n"/>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="15" t="n"/>
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>Mining Investigations</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="n"/>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="15" t="n"/>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>Firearm Training</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="n"/>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="15" t="n"/>
+      <c r="B38" s="17" t="inlineStr">
+        <is>
+          <t>Corporate Training</t>
+        </is>
+      </c>
+      <c r="C38" s="19" t="n"/>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="15" t="n"/>
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>Riot Control Training</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="n"/>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="15" t="n"/>
+      <c r="B40" s="17" t="inlineStr">
+        <is>
+          <t>Security Training</t>
+        </is>
+      </c>
+      <c r="C40" s="19" t="n"/>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="15" t="n"/>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>Bespoke risk solutions</t>
+        </is>
+      </c>
+      <c r="C41" s="19" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C6 C7 C8 C9 C10 C11 C12 C14 C16 C17 C18 C20 C21 C22 C23 C25 C26 C27 C28 C30 C32 C33 C34 C35 C36 C37 C38 C39 C40 C41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"YES,NO"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2203,7 +2609,7 @@
           <t>INTEGRI Forensic Services (Pty) Ltd</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Confirmed from CIPC certificate</t>
         </is>
@@ -2220,7 +2626,7 @@
           <t>2026/561988/07</t>
         </is>
       </c>
-      <c r="C6" s="21" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Confirmed from CIPC certificate</t>
         </is>
@@ -2237,7 +2643,7 @@
           <t>INTEGRI Forensic and Protection Services</t>
         </is>
       </c>
-      <c r="C7" s="21" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>Confirmed</t>
         </is>
@@ -2249,8 +2655,8 @@
           <t>PSIRA registration number (business)</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr"/>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr"/>
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Needed — attach the certificate</t>
         </is>
@@ -2262,8 +2668,8 @@
           <t>PSIRA registration expiry / renewal date</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr"/>
-      <c r="C9" s="21" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr"/>
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Needed</t>
         </is>
@@ -2275,8 +2681,8 @@
           <t>VAT number (if registered)</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr"/>
-      <c r="C10" s="21" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr"/>
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>Leave blank if not VAT registered</t>
         </is>
@@ -2288,8 +2694,8 @@
           <t>Firearm training accreditation body</t>
         </is>
       </c>
-      <c r="B11" s="19" t="inlineStr"/>
-      <c r="C11" s="21" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr"/>
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>e.g. SAPS, SASSETA</t>
         </is>
@@ -2301,8 +2707,8 @@
           <t>Firearm training accreditation number</t>
         </is>
       </c>
-      <c r="B12" s="19" t="inlineStr"/>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr"/>
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>Needed — attach the certificate</t>
         </is>
@@ -2314,8 +2720,8 @@
           <t>Firearm competency types covered</t>
         </is>
       </c>
-      <c r="B13" s="19" t="inlineStr"/>
-      <c r="C13" s="21" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr"/>
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>e.g. handgun, shotgun, rifle, self-defence, business purposes</t>
         </is>
@@ -2327,8 +2733,8 @@
           <t>B-BBEE level</t>
         </is>
       </c>
-      <c r="B14" s="19" t="inlineStr"/>
-      <c r="C14" s="21" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr"/>
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Leave blank if not yet assessed</t>
         </is>
@@ -2340,8 +2746,8 @@
           <t>Business address to publish on the site</t>
         </is>
       </c>
-      <c r="B15" s="19" t="inlineStr"/>
-      <c r="C15" s="21" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr"/>
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>The CIPC address is residential and is NOT published. Give a commercial or PO Box address, or write NONE.</t>
         </is>
@@ -2353,8 +2759,8 @@
           <t>Office hours (admin and quotes)</t>
         </is>
       </c>
-      <c r="B16" s="19" t="inlineStr"/>
-      <c r="C16" s="21" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr"/>
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>e.g. Mon-Fri 08:00-17:00</t>
         </is>
@@ -2366,8 +2772,8 @@
           <t>After-hours / emergency availability</t>
         </is>
       </c>
-      <c r="B17" s="19" t="inlineStr"/>
-      <c r="C17" s="21" t="inlineStr">
+      <c r="B17" s="20" t="inlineStr"/>
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>Is the 24/7 line genuinely answered at any hour?</t>
         </is>
@@ -2379,8 +2785,8 @@
           <t>Provinces actually serviced</t>
         </is>
       </c>
-      <c r="B18" s="19" t="inlineStr"/>
-      <c r="C18" s="21" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr"/>
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>The site currently says 'national'. List the real provinces.</t>
         </is>
@@ -2392,8 +2798,8 @@
           <t>Website domain registered to INTEGRI?</t>
         </is>
       </c>
-      <c r="B19" s="19" t="inlineStr"/>
-      <c r="C19" s="21" t="inlineStr">
+      <c r="B19" s="20" t="inlineStr"/>
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>Yes / No</t>
         </is>
@@ -2405,8 +2811,8 @@
           <t>Is ops@ ... .com live and monitored?</t>
         </is>
       </c>
-      <c r="B20" s="19" t="inlineStr"/>
-      <c r="C20" s="21" t="inlineStr">
+      <c r="B20" s="20" t="inlineStr"/>
+      <c r="C20" s="18" t="inlineStr">
         <is>
           <t>Yes / No</t>
         </is>
@@ -2418,8 +2824,8 @@
           <t>LinkedIn URL</t>
         </is>
       </c>
-      <c r="B21" s="19" t="inlineStr"/>
-      <c r="C21" s="21" t="inlineStr">
+      <c r="B21" s="20" t="inlineStr"/>
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t>Leave blank if none</t>
         </is>
@@ -2431,8 +2837,8 @@
           <t>Facebook URL</t>
         </is>
       </c>
-      <c r="B22" s="19" t="inlineStr"/>
-      <c r="C22" s="21" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr"/>
+      <c r="C22" s="18" t="inlineStr">
         <is>
           <t>Leave blank if none</t>
         </is>
@@ -2444,8 +2850,8 @@
           <t>Instagram URL</t>
         </is>
       </c>
-      <c r="B23" s="19" t="inlineStr"/>
-      <c r="C23" s="21" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr"/>
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t>Leave blank if none</t>
         </is>
@@ -2457,8 +2863,8 @@
           <t>Professional indemnity insurer &amp; cover</t>
         </is>
       </c>
-      <c r="B24" s="19" t="inlineStr"/>
-      <c r="C24" s="21" t="inlineStr">
+      <c r="B24" s="20" t="inlineStr"/>
+      <c r="C24" s="18" t="inlineStr">
         <is>
           <t>Not published — used when clients ask</t>
         </is>
@@ -2470,8 +2876,8 @@
           <t>Public liability insurer &amp; cover</t>
         </is>
       </c>
-      <c r="B25" s="19" t="inlineStr"/>
-      <c r="C25" s="21" t="inlineStr">
+      <c r="B25" s="20" t="inlineStr"/>
+      <c r="C25" s="18" t="inlineStr">
         <is>
           <t>Not published — used when clients ask</t>
         </is>
@@ -2486,7 +2892,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2549,10 +2955,10 @@
           <t>Etienne</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n"/>
-      <c r="C5" s="19" t="n"/>
-      <c r="D5" s="19" t="n"/>
-      <c r="E5" s="21" t="inlineStr">
+      <c r="B5" s="20" t="n"/>
+      <c r="C5" s="20" t="n"/>
+      <c r="D5" s="20" t="n"/>
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>The site currently says 'Director'. CIPC lists only Anri Coetser as a director — give the correct title.</t>
         </is>
@@ -2564,10 +2970,10 @@
           <t>Jacques</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n"/>
-      <c r="C6" s="19" t="n"/>
-      <c r="D6" s="19" t="n"/>
-      <c r="E6" s="21" t="inlineStr">
+      <c r="B6" s="20" t="n"/>
+      <c r="C6" s="20" t="n"/>
+      <c r="D6" s="20" t="n"/>
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>The site currently says 'Director'. Give the correct title.</t>
         </is>
@@ -2579,10 +2985,10 @@
           <t>Anri Coetser</t>
         </is>
       </c>
-      <c r="B7" s="19" t="n"/>
-      <c r="C7" s="19" t="n"/>
-      <c r="D7" s="19" t="n"/>
-      <c r="E7" s="21" t="inlineStr">
+      <c r="B7" s="20" t="n"/>
+      <c r="C7" s="20" t="n"/>
+      <c r="D7" s="20" t="n"/>
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>Sole CIPC-registered director. Should she appear on the website at all? Yes / No.</t>
         </is>
@@ -2594,10 +3000,10 @@
           <t>Information Officer</t>
         </is>
       </c>
-      <c r="B8" s="19" t="n"/>
-      <c r="C8" s="19" t="n"/>
-      <c r="D8" s="19" t="n"/>
-      <c r="E8" s="21" t="inlineStr">
+      <c r="B8" s="20" t="n"/>
+      <c r="C8" s="20" t="n"/>
+      <c r="D8" s="20" t="n"/>
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>Required by POPIA because the website collects enquiries. Usually a director. Must be registered with the Information Regulator.</t>
         </is>
@@ -2609,10 +3015,10 @@
           <t>Deputy Information Officer</t>
         </is>
       </c>
-      <c r="B9" s="19" t="n"/>
-      <c r="C9" s="19" t="n"/>
-      <c r="D9" s="19" t="n"/>
-      <c r="E9" s="21" t="inlineStr">
+      <c r="B9" s="20" t="n"/>
+      <c r="C9" s="20" t="n"/>
+      <c r="D9" s="20" t="n"/>
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>Optional.</t>
         </is>
@@ -2624,10 +3030,10 @@
           <t>Polygraph examiner</t>
         </is>
       </c>
-      <c r="B10" s="19" t="n"/>
-      <c r="C10" s="19" t="n"/>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="21" t="inlineStr">
+      <c r="B10" s="20" t="n"/>
+      <c r="C10" s="20" t="n"/>
+      <c r="D10" s="20" t="n"/>
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>Backs the polygraph pages.</t>
         </is>
@@ -2639,10 +3045,10 @@
           <t>Firearm instructor</t>
         </is>
       </c>
-      <c r="B11" s="19" t="n"/>
-      <c r="C11" s="19" t="n"/>
-      <c r="D11" s="19" t="n"/>
-      <c r="E11" s="21" t="inlineStr">
+      <c r="B11" s="20" t="n"/>
+      <c r="C11" s="20" t="n"/>
+      <c r="D11" s="20" t="n"/>
+      <c r="E11" s="18" t="inlineStr">
         <is>
           <t>Backs the firearm training claim.</t>
         </is>
@@ -2654,17 +3060,17 @@
           <t>Forensic expert witness</t>
         </is>
       </c>
-      <c r="B12" s="19" t="n"/>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="21" t="inlineStr">
+      <c r="B12" s="20" t="n"/>
+      <c r="C12" s="20" t="n"/>
+      <c r="D12" s="20" t="n"/>
+      <c r="E12" s="18" t="inlineStr">
         <is>
           <t>The site offers expert witness testimony — who would actually testify?</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>Do NOT include ID numbers or home addresses — we do not publish them and do not need them.</t>
         </is>
@@ -2679,7 +3085,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2739,12 +3145,12 @@
           <t>PSIRA registration certificate — business</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Publishes the registration number and supports the compliance statement on every page</t>
         </is>
       </c>
-      <c r="D5" s="18" t="n"/>
+      <c r="D5" s="19" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="14" t="n">
@@ -2755,12 +3161,12 @@
           <t>PSIRA certificates — individual officers</t>
         </is>
       </c>
-      <c r="C6" s="21" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>The guarding and protection pages state officers are registered and graded</t>
         </is>
       </c>
-      <c r="D6" s="18" t="n"/>
+      <c r="D6" s="19" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="14" t="n">
@@ -2771,12 +3177,12 @@
           <t>Firearm training accreditation certificate</t>
         </is>
       </c>
-      <c r="C7" s="21" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>Supports the accredited firearm training claim</t>
         </is>
       </c>
-      <c r="D7" s="18" t="n"/>
+      <c r="D7" s="19" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="14" t="n">
@@ -2787,12 +3193,12 @@
           <t>Polygraph examiner qualification(s)</t>
         </is>
       </c>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Supports the polygraph division</t>
         </is>
       </c>
-      <c r="D8" s="18" t="n"/>
+      <c r="D8" s="19" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="14" t="n">
@@ -2803,12 +3209,12 @@
           <t>Tax clearance certificate</t>
         </is>
       </c>
-      <c r="C9" s="21" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Corporate clients and tenders</t>
         </is>
       </c>
-      <c r="D9" s="18" t="n"/>
+      <c r="D9" s="19" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="14" t="n">
@@ -2819,12 +3225,12 @@
           <t>VAT registration certificate</t>
         </is>
       </c>
-      <c r="C10" s="21" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>Only if VAT registered — for the footer</t>
         </is>
       </c>
-      <c r="D10" s="18" t="n"/>
+      <c r="D10" s="19" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="14" t="n">
@@ -2835,12 +3241,12 @@
           <t>B-BBEE certificate or sworn affidavit</t>
         </is>
       </c>
-      <c r="C11" s="21" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>Tenders and corporate procurement</t>
         </is>
       </c>
-      <c r="D11" s="18" t="n"/>
+      <c r="D11" s="19" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="14" t="n">
@@ -2851,12 +3257,12 @@
           <t>Professional indemnity insurance schedule</t>
         </is>
       </c>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>Clients ask before appointing</t>
         </is>
       </c>
-      <c r="D12" s="18" t="n"/>
+      <c r="D12" s="19" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="14" t="n">
@@ -2867,12 +3273,12 @@
           <t>Public liability insurance schedule</t>
         </is>
       </c>
-      <c r="C13" s="21" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>Clients ask before appointing</t>
         </is>
       </c>
-      <c r="D13" s="18" t="n"/>
+      <c r="D13" s="19" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="14" t="n">
@@ -2883,12 +3289,12 @@
           <t>Company letterhead / brand guide</t>
         </is>
       </c>
-      <c r="C14" s="21" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Keeps documents consistent with the site</t>
         </is>
       </c>
-      <c r="D14" s="18" t="n"/>
+      <c r="D14" s="19" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="14" t="n">
@@ -2899,12 +3305,12 @@
           <t>Logo — full lockup, transparent PNG</t>
         </is>
       </c>
-      <c r="C15" s="21" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>Crest received. Lockup with wordmark still wanted for documents.</t>
         </is>
       </c>
-      <c r="D15" s="18" t="n"/>
+      <c r="D15" s="19" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="14" t="n">
@@ -2915,12 +3321,12 @@
           <t>Team photographs (optional)</t>
         </is>
       </c>
-      <c r="C16" s="21" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>Would replace the initial-letter avatars on the site</t>
         </is>
       </c>
-      <c r="D16" s="18" t="n"/>
+      <c r="D16" s="19" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="14" t="n">
@@ -2931,12 +3337,12 @@
           <t>CIPC registration certificate</t>
         </is>
       </c>
-      <c r="C17" s="21" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>RECEIVED — no action needed</t>
         </is>
       </c>
-      <c r="D17" s="23" t="inlineStr">
+      <c r="D17" s="24" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2951,12 +3357,12 @@
           <t>Logo — crest, transparent PNG</t>
         </is>
       </c>
-      <c r="C18" s="21" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>RECEIVED — now live on the site</t>
         </is>
       </c>
-      <c r="D18" s="23" t="inlineStr">
+      <c r="D18" s="24" t="inlineStr">
         <is>
           <t>YES</t>
         </is>

</xml_diff>